<commit_message>
Updated RAD Existing Test Cases for Notice Number Verbiage
</commit_message>
<xml_diff>
--- a/KatalonData/RADTestData/ContinueButton.xlsx
+++ b/KatalonData/RADTestData/ContinueButton.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\RADTestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E964A0-4BFC-43E0-98D6-3C2B36758A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903F84FE-D89C-43A4-9FC7-1BB76E04664E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5018" yWindow="3157" windowWidth="21600" windowHeight="11326" firstSheet="1" activeTab="6" xr2:uid="{D99FAB39-5CE6-4AA4-B9C6-99B1EFA0654E}"/>
+    <workbookView xWindow="6180" yWindow="2160" windowWidth="21600" windowHeight="11325" firstSheet="1" activeTab="6" xr2:uid="{D99FAB39-5CE6-4AA4-B9C6-99B1EFA0654E}"/>
   </bookViews>
   <sheets>
     <sheet name="Estimated" sheetId="1" r:id="rId1"/>
@@ -233,319 +233,319 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>Fri Oct 02 20:30:58 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:31:29 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:31:47 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:32:33 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:32:48 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:33:06 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:33:27 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:33:43 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:33:59 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:34:14 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:34:31 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:34:46 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:35:03 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:35:21 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:35:37 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:35:54 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:36:09 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:36:25 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:36:40 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:36:55 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:37:11 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:37:26 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:39:07 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:39:21 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:39:36 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:39:52 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:40:14 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:40:36 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:40:57 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:41:18 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:41:39 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:42:00 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:42:21 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:42:41 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:43:07 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:43:29 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:43:50 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:44:11 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:44:33 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:44:54 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:45:15 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:45:37 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:45:59 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:46:19 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:46:40 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:47:01 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:47:21 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:47:42 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:48:03 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:48:25 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:48:47 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:49:08 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:49:30 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:49:51 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:50:12 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:50:33 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:50:54 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:51:15 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:51:36 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:51:58 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:52:19 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:52:41 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:53:02 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:53:28 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:53:49 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:54:09 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:54:30 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:54:52 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:55:13 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:55:35 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:55:56 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:56:18 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:56:39 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:57:00 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:57:22 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:57:43 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:58:04 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:58:24 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:58:45 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:59:05 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:59:26 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 20:59:47 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:00:09 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:00:31 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:00:53 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:01:14 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:01:28 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:01:44 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:01:59 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:02:14 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:02:29 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:02:44 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:03:00 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:03:15 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:03:31 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:03:59 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:04:26 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:04:53 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:05:20 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:13:14 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:13:32 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:14:02 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:14:20 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:14:36 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Oct 02 21:16:20 EDT 2026</t>
+    <t>Tue Oct 27 16:52:08 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:52:31 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:52:50 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:53:24 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:53:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:54:13 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:54:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:54:50 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:55:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:55:23 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:55:40 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:55:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:56:14 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:56:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:56:51 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:57:08 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:57:25 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:57:41 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:58:21 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:58:42 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:58:59 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:59:16 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:59:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 16:59:55 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:01:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:02:48 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:03:05 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:03:22 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:03:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:04:09 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:04:31 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:04:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:05:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:05:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:06:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:06:25 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:06:48 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:07:10 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:07:32 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:07:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:08:16 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:08:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:09:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:09:25 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:09:48 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:10:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:10:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:10:57 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:11:20 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:11:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:12:06 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:12:29 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:12:52 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:13:15 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:13:38 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:14:00 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:14:23 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:14:46 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:15:08 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:15:32 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:15:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:16:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:16:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:17:03 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:17:26 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:17:48 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:18:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:18:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:18:57 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:19:19 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:19:42 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:20:06 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:20:28 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:20:51 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:21:14 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:21:37 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:22:00 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:22:23 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:22:46 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:23:09 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:23:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:23:56 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:24:19 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:24:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:25:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:25:30 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:25:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:26:16 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:26:32 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:26:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:27:06 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:27:22 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:27:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:27:55 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:28:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:28:28 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:28:45 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:29:14 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:29:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:30:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 17:30:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 21:02:26 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 21:04:13 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 21:04:32 EDT 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 21:07:25 EDT 2026</t>
   </si>
 </sst>
 </file>
@@ -967,7 +967,7 @@
         <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>161</v>
+        <v>62</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>
@@ -993,7 +993,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>29</v>
@@ -1019,7 +1019,7 @@
         <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>162</v>
+        <v>64</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>29</v>
@@ -1045,7 +1045,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>163</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>29</v>
@@ -1071,7 +1071,7 @@
         <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>29</v>
@@ -1097,7 +1097,7 @@
         <v>61</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>166</v>
+        <v>66</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>29</v>
@@ -1123,7 +1123,7 @@
         <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>163</v>
+        <v>67</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>29</v>
@@ -1199,7 +1199,7 @@
         <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>
@@ -1219,7 +1219,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>29</v>
@@ -1239,7 +1239,7 @@
         <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>29</v>
@@ -1259,7 +1259,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>29</v>
@@ -1279,7 +1279,7 @@
         <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>29</v>
@@ -1299,7 +1299,7 @@
         <v>61</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>29</v>
@@ -1322,7 +1322,7 @@
         <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>29</v>
@@ -1345,7 +1345,7 @@
         <v>61</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>29</v>
@@ -1368,7 +1368,7 @@
         <v>61</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>29</v>
@@ -1391,7 +1391,7 @@
         <v>61</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>29</v>
@@ -1411,7 +1411,7 @@
         <v>61</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>29</v>
@@ -1431,7 +1431,7 @@
         <v>61</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>29</v>
@@ -1454,7 +1454,7 @@
         <v>61</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>29</v>
@@ -1477,7 +1477,7 @@
         <v>61</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>29</v>
@@ -1497,7 +1497,7 @@
         <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>29</v>
@@ -1520,7 +1520,7 @@
         <v>61</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>29</v>
@@ -1543,7 +1543,7 @@
         <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>29</v>
@@ -1577,7 +1577,7 @@
         <v>61</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>29</v>
@@ -1668,7 +1668,7 @@
         <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>
@@ -1694,7 +1694,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>29</v>
@@ -1717,7 +1717,7 @@
         <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>165</v>
+        <v>86</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>29</v>
@@ -1740,7 +1740,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>84</v>
+        <v>166</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>29</v>
@@ -1763,7 +1763,7 @@
         <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>29</v>
@@ -1786,7 +1786,7 @@
         <v>61</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>29</v>
@@ -1873,7 +1873,7 @@
         <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>
@@ -1896,7 +1896,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>29</v>
@@ -1919,7 +1919,7 @@
         <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>29</v>
@@ -1942,7 +1942,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>29</v>
@@ -1965,7 +1965,7 @@
         <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>29</v>
@@ -1988,7 +1988,7 @@
         <v>61</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>29</v>
@@ -2011,7 +2011,7 @@
         <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>29</v>
@@ -2034,7 +2034,7 @@
         <v>61</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>29</v>
@@ -2057,7 +2057,7 @@
         <v>61</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>29</v>
@@ -2080,7 +2080,7 @@
         <v>61</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>29</v>
@@ -2103,7 +2103,7 @@
         <v>61</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>29</v>
@@ -2126,7 +2126,7 @@
         <v>61</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>29</v>
@@ -2149,7 +2149,7 @@
         <v>61</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>29</v>
@@ -2172,7 +2172,7 @@
         <v>61</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>29</v>
@@ -2195,7 +2195,7 @@
         <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>29</v>
@@ -2218,7 +2218,7 @@
         <v>61</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>29</v>
@@ -2247,7 +2247,7 @@
         <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>29</v>
@@ -2276,7 +2276,7 @@
         <v>61</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>29</v>
@@ -2305,7 +2305,7 @@
         <v>61</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>29</v>
@@ -2328,7 +2328,7 @@
         <v>61</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>29</v>
@@ -2357,7 +2357,7 @@
         <v>61</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>29</v>
@@ -2386,7 +2386,7 @@
         <v>61</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>29</v>
@@ -2412,7 +2412,7 @@
         <v>61</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>29</v>
@@ -2441,7 +2441,7 @@
         <v>61</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>29</v>
@@ -2470,7 +2470,7 @@
         <v>61</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>29</v>
@@ -2499,7 +2499,7 @@
         <v>61</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>29</v>
@@ -2525,7 +2525,7 @@
         <v>61</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>29</v>
@@ -2554,7 +2554,7 @@
         <v>61</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>29</v>
@@ -2583,7 +2583,7 @@
         <v>61</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>29</v>
@@ -2612,7 +2612,7 @@
         <v>61</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>29</v>
@@ -2641,7 +2641,7 @@
         <v>61</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>29</v>
@@ -2664,7 +2664,7 @@
         <v>61</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>29</v>
@@ -2693,7 +2693,7 @@
         <v>61</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>29</v>
@@ -2722,7 +2722,7 @@
         <v>61</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>29</v>
@@ -2748,7 +2748,7 @@
         <v>61</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>29</v>
@@ -2777,7 +2777,7 @@
         <v>61</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>29</v>
@@ -2806,7 +2806,7 @@
         <v>61</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>29</v>
@@ -2835,7 +2835,7 @@
         <v>61</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>29</v>
@@ -2861,7 +2861,7 @@
         <v>61</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>29</v>
@@ -2890,7 +2890,7 @@
         <v>61</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>29</v>
@@ -2919,7 +2919,7 @@
         <v>61</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>29</v>
@@ -2948,7 +2948,7 @@
         <v>61</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>29</v>
@@ -2977,7 +2977,7 @@
         <v>61</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>29</v>
@@ -3000,7 +3000,7 @@
         <v>61</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>29</v>
@@ -3029,7 +3029,7 @@
         <v>61</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>29</v>
@@ -3058,7 +3058,7 @@
         <v>61</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>29</v>
@@ -3084,7 +3084,7 @@
         <v>61</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>29</v>
@@ -3113,7 +3113,7 @@
         <v>61</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>29</v>
@@ -3142,7 +3142,7 @@
         <v>61</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>29</v>
@@ -3171,7 +3171,7 @@
         <v>61</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>29</v>
@@ -3197,7 +3197,7 @@
         <v>61</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>29</v>
@@ -3226,7 +3226,7 @@
         <v>61</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>29</v>
@@ -3249,7 +3249,7 @@
         <v>61</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>29</v>
@@ -3295,7 +3295,7 @@
         <v>61</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>29</v>
@@ -3318,7 +3318,7 @@
         <v>61</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>29</v>
@@ -3364,7 +3364,7 @@
         <v>61</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>29</v>
@@ -3387,7 +3387,7 @@
         <v>61</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>29</v>
@@ -3433,7 +3433,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>29</v>
@@ -3459,7 +3459,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>29</v>
@@ -3485,7 +3485,7 @@
         <v>61</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>29</v>
@@ -3554,7 +3554,7 @@
         <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>
@@ -3574,7 +3574,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>29</v>
@@ -3594,7 +3594,7 @@
         <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>29</v>
@@ -3614,7 +3614,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>29</v>
@@ -3634,7 +3634,7 @@
         <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>29</v>
@@ -3654,7 +3654,7 @@
         <v>61</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>29</v>
@@ -3674,7 +3674,7 @@
         <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>29</v>
@@ -3694,7 +3694,7 @@
         <v>61</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>29</v>
@@ -3752,7 +3752,7 @@
         <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>
@@ -3772,7 +3772,7 @@
         <v>61</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>29</v>
@@ -3792,7 +3792,7 @@
         <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>29</v>
@@ -3812,7 +3812,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>29</v>
@@ -3832,7 +3832,7 @@
         <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>29</v>
@@ -3887,7 +3887,7 @@
         <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>

</xml_diff>